<commit_message>
Resources: PROG-WT carries SAR value at price 1, COST-SAR price 0 (EV/CPI/SPI in SAR on progress distribution)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DZdGPWRxvKXCnMyT6qFPZb
</commit_message>
<xml_diff>
--- a/p6/SAR_BOQ_Cost_Mapping.xlsx
+++ b/p6/SAR_BOQ_Cost_Mapping.xlsx
@@ -60437,16 +60437,16 @@
         </is>
       </c>
       <c r="E2" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>Budgeted cost of the activity in SAR from the contract payment conditions applied to the BOQ station value</t>
+          <t>Contract cost of the activity in SAR from the payment conditions applied to the BOQ station value (column L of BOQ_Mapping)</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>Material resource: cost only. Budgeted units = SAR, so budgeted cost = units x 1. Not counted in Units % complete.</t>
+          <t>Quantity carrier. Price 0, so it adds no budget cost. Set the price to 1 (and PROG-WT to 0) to see the contract-condition cost curve instead.</t>
         </is>
       </c>
     </row>
@@ -60458,7 +60458,7 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Progress weight (fair EPC distribution)</t>
+          <t>Progress weight (fair EPC distribution, SAR value)</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -60468,20 +60468,20 @@
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>SAR</t>
         </is>
       </c>
       <c r="E3" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>Progress points: 100,000 points = 100% of the project. Fair EPC distribution (see Distribution_Keys)</t>
+          <t>Progress share x SAR 62,000,000 (100,000 points x SAR 620). Fair EPC distribution (see Distribution_Keys)</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>Nonlabor resource with zero price. Activity % complete type is Units, so P6 measures progress with these points and the S-curve follows the points</t>
+          <t>Price 1, so budgeted cost = progress value in SAR. Activity % complete type is Physical, so earned value = physical % x this budget, and the cost and schedule performance indexes are measured in SAR on the progress distribution.</t>
         </is>
       </c>
     </row>

</xml_diff>